<commit_message>
Fixing xlwings in calibration script and fixing xlsx dependencies for auto ownership
</commit_message>
<xml_diff>
--- a/utilities/calibration/workbook_templates/02_AutoOwnership_2023_blank.xlsx
+++ b/utilities/calibration/workbook_templates/02_AutoOwnership_2023_blank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one\utilities\calibration\workbook_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D245E3F-F611-4129-8011-B56D4B87968D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC053FE-9649-4243-AAD0-DA750F063B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="3" r:id="rId1"/>
@@ -5268,25 +5268,25 @@
       <c r="I5" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="J5" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K5" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L5" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M5" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N5" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
+      <c r="J5" s="14">
+        <f>summary!C31</f>
+        <v>9.8525035397454774E-2</v>
+      </c>
+      <c r="K5" s="14">
+        <f>summary!D31</f>
+        <v>0.33424947504373459</v>
+      </c>
+      <c r="L5" s="14">
+        <f>summary!E31</f>
+        <v>0.3465181198228573</v>
+      </c>
+      <c r="M5" s="14">
+        <f>summary!F31</f>
+        <v>0.13919218910295361</v>
+      </c>
+      <c r="N5" s="14">
+        <f>summary!G31</f>
+        <v>8.1515180632999756E-2</v>
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.2">
@@ -5358,25 +5358,25 @@
       <c r="I7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J7" s="14" t="e">
+      <c r="J7" s="14">
         <f t="shared" ref="J7:N7" si="0">J6-J5</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K7" s="14" t="e">
+        <v>0.10147496460254524</v>
+      </c>
+      <c r="K7" s="14">
         <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="L7" s="14" t="e">
+        <v>-0.13424947504373458</v>
+      </c>
+      <c r="L7" s="14">
         <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="M7" s="14" t="e">
+        <v>-0.14651811982285728</v>
+      </c>
+      <c r="M7" s="14">
         <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="N7" s="14" t="e">
+        <v>6.0807810897046399E-2</v>
+      </c>
+      <c r="N7" s="14">
         <f t="shared" si="0"/>
-        <v>#REF!</v>
+        <v>0.11848481936700025</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
@@ -5405,25 +5405,25 @@
       <c r="I8" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="J8" s="16" t="e">
+      <c r="J8" s="16">
         <f t="shared" ref="J8:N8" si="1">J7/J5</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K8" s="16" t="e">
+        <v>1.0299409098732144</v>
+      </c>
+      <c r="K8" s="16">
         <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="L8" s="16" t="e">
+        <v>-0.40164453519685805</v>
+      </c>
+      <c r="L8" s="16">
         <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="M8" s="16" t="e">
+        <v>-0.42282960526785285</v>
+      </c>
+      <c r="M8" s="16">
         <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="N8" s="16" t="e">
+        <v>0.43686223550999587</v>
+      </c>
+      <c r="N8" s="16">
         <f t="shared" si="1"/>
-        <v>#REF!</v>
+        <v>1.4535307220926907</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
@@ -5526,21 +5526,21 @@
       <c r="J11" s="19">
         <v>0</v>
       </c>
-      <c r="K11" s="20" t="e">
+      <c r="K11" s="20">
         <f>damp*LN(K5/K6)-damp*LN($J5/$J6)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L11" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="L11" s="20">
         <f>damp*LN(L5/L6)-damp*LN($J5/$J6)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M11" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="M11" s="20">
         <f>damp*LN(M5/M6)-damp*LN($J5/$J6)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N11" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="N11" s="20">
         <f>damp*LN(N5/N6)-damp*LN($J5/$J6)</f>
-        <v>#REF!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.2">
@@ -5573,21 +5573,21 @@
         <f>J10+J11</f>
         <v>0</v>
       </c>
-      <c r="K12" s="21" t="e">
+      <c r="K12" s="21">
         <f>K10+K11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L12" s="21" t="e">
+        <v>1.1172992162790916</v>
+      </c>
+      <c r="L12" s="21">
         <f>L10+L11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M12" s="21" t="e">
+        <v>-1.2565051850306308</v>
+      </c>
+      <c r="M12" s="21">
         <f>M10+M11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N12" s="21" t="e">
+        <v>-3.3877106944960214</v>
+      </c>
+      <c r="N12" s="21">
         <f>N10+N11</f>
-        <v>#REF!</v>
+        <v>-5.3502031433147499</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.2">
@@ -5683,44 +5683,44 @@
       <c r="C18" s="25">
         <v>0</v>
       </c>
-      <c r="D18" s="33" t="e">
+      <c r="D18" s="33">
         <f>K12</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E18" s="33" t="e">
+        <v>1.1172992162790916</v>
+      </c>
+      <c r="E18" s="33">
         <f>L12</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F18" s="33" t="e">
+        <v>-1.2565051850306308</v>
+      </c>
+      <c r="F18" s="33">
         <f>M12</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G18" s="33" t="e">
+        <v>-3.3877106944960214</v>
+      </c>
+      <c r="G18" s="33">
         <f>N12</f>
-        <v>#REF!</v>
+        <v>-5.3502031433147499</v>
       </c>
       <c r="I18" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="J18" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K18" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L18" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M18" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N18" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
+      <c r="J18" s="14">
+        <f>summary!C22</f>
+        <v>0.30941840242778079</v>
+      </c>
+      <c r="K18" s="14">
+        <f>summary!D22</f>
+        <v>0.43931757641246466</v>
+      </c>
+      <c r="L18" s="14">
+        <f>summary!E22</f>
+        <v>0.19018512097240253</v>
+      </c>
+      <c r="M18" s="14">
+        <f>summary!F22</f>
+        <v>3.9894953860875687E-2</v>
+      </c>
+      <c r="N18" s="14">
+        <f>summary!G22</f>
+        <v>2.1183946326476303E-2</v>
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.2">
@@ -5730,21 +5730,21 @@
       <c r="C19" s="24">
         <v>0</v>
       </c>
-      <c r="D19" s="33" t="e">
+      <c r="D19" s="33">
         <f>K25</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E19" s="33" t="e">
+        <v>0.57931801393948956</v>
+      </c>
+      <c r="E19" s="33">
         <f>L25</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F19" s="33" t="e">
+        <v>0.56301198136124597</v>
+      </c>
+      <c r="F19" s="33">
         <f>M25</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G19" s="33" t="e">
+        <v>0.4050938414636639</v>
+      </c>
+      <c r="G19" s="33">
         <f>N25</f>
-        <v>#REF!</v>
+        <v>-0.20245078944536879</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>42</v>
@@ -5792,25 +5792,25 @@
       <c r="I20" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J20" s="14" t="e">
+      <c r="J20" s="14">
         <f>J19-J18</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K20" s="14" t="e">
+        <v>-0.10941840242778078</v>
+      </c>
+      <c r="K20" s="14">
         <f>K19-K18</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L20" s="14" t="e">
+        <v>-0.23931757641246465</v>
+      </c>
+      <c r="L20" s="14">
         <f>L19-L18</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M20" s="14" t="e">
+        <v>9.8148790275974784E-3</v>
+      </c>
+      <c r="M20" s="14">
         <f>M19-M18</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N20" s="14" t="e">
+        <v>0.16010504613912432</v>
+      </c>
+      <c r="N20" s="14">
         <f>N19-N18</f>
-        <v>#REF!</v>
+        <v>0.17881605367352371</v>
       </c>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.2">
@@ -5821,44 +5821,44 @@
         <f>J61</f>
         <v>0</v>
       </c>
-      <c r="D21" s="33" t="e">
+      <c r="D21" s="33">
         <f>K61</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E21" s="33" t="e">
+        <v>0.1844471057264194</v>
+      </c>
+      <c r="E21" s="33">
         <f t="shared" ref="E21:G21" si="3">L61</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F21" s="33" t="e">
+        <v>0.1844471057264194</v>
+      </c>
+      <c r="F21" s="33">
         <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G21" s="33" t="e">
+        <v>0.20643155178083641</v>
+      </c>
+      <c r="G21" s="33">
         <f t="shared" si="3"/>
-        <v>#REF!</v>
+        <v>0.20643155178083641</v>
       </c>
       <c r="I21" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="J21" s="16" t="e">
+      <c r="J21" s="16">
         <f>J20/J18</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K21" s="16" t="e">
+        <v>-0.35362603377580093</v>
+      </c>
+      <c r="K21" s="16">
         <f>K20/K18</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L21" s="16" t="e">
+        <v>-0.54474846730870419</v>
+      </c>
+      <c r="L21" s="16">
         <f>L20/L18</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M21" s="16" t="e">
+        <v>5.1606976284026447E-2</v>
+      </c>
+      <c r="M21" s="16">
         <f>M20/M18</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N21" s="16" t="e">
+        <v>4.0131653415981683</v>
+      </c>
+      <c r="N21" s="16">
         <f>N20/N18</f>
-        <v>#REF!</v>
+        <v>8.4411115340692824</v>
       </c>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.2">
@@ -5936,21 +5936,21 @@
         <f>J37</f>
         <v>0</v>
       </c>
-      <c r="D24" s="33" t="e">
+      <c r="D24" s="33">
         <f>K37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E24" s="33" t="e">
+        <v>-0.57903681911096483</v>
+      </c>
+      <c r="E24" s="33">
         <f>L37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F24" s="33" t="e">
+        <v>-0.3943306525851169</v>
+      </c>
+      <c r="F24" s="33">
         <f>M37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G24" s="33" t="e">
+        <v>-0.20319232197177453</v>
+      </c>
+      <c r="G24" s="33">
         <f>N37</f>
-        <v>#REF!</v>
+        <v>-4.5351682239474958E-2</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>53</v>
@@ -5958,21 +5958,21 @@
       <c r="J24" s="19">
         <v>0</v>
       </c>
-      <c r="K24" s="20" t="e">
+      <c r="K24" s="20">
         <f>damp*LN(K18/K19)-damp*LN($J18/$J19)-K11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L24" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="L24" s="20">
         <f>damp*LN(L18/L19)-damp*LN($J18/$J19)-L11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M24" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="M24" s="20">
         <f>damp*LN(M18/M19)-damp*LN($J18/$J19)-M11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N24" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="N24" s="20">
         <f>damp*LN(N18/N19)-damp*LN($J18/$J19)</f>
-        <v>#REF!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -5983,21 +5983,21 @@
         <f>J37</f>
         <v>0</v>
       </c>
-      <c r="D25" s="33" t="e">
+      <c r="D25" s="33">
         <f>K37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E25" s="33" t="e">
+        <v>-0.57903681911096483</v>
+      </c>
+      <c r="E25" s="33">
         <f>L37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F25" s="33" t="e">
+        <v>-0.3943306525851169</v>
+      </c>
+      <c r="F25" s="33">
         <f>M37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G25" s="33" t="e">
+        <v>-0.20319232197177453</v>
+      </c>
+      <c r="G25" s="33">
         <f>N37</f>
-        <v>#REF!</v>
+        <v>-4.5351682239474958E-2</v>
       </c>
       <c r="I25" s="18" t="s">
         <v>59</v>
@@ -6006,21 +6006,21 @@
         <f>J23+J24</f>
         <v>0</v>
       </c>
-      <c r="K25" s="21" t="e">
+      <c r="K25" s="21">
         <f>K23+K24</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L25" s="21" t="e">
+        <v>0.57931801393948956</v>
+      </c>
+      <c r="L25" s="21">
         <f>L23+L24</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M25" s="21" t="e">
+        <v>0.56301198136124597</v>
+      </c>
+      <c r="M25" s="21">
         <f>M23+M24</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N25" s="21" t="e">
+        <v>0.4050938414636639</v>
+      </c>
+      <c r="N25" s="21">
         <f>N23+N24</f>
-        <v>#REF!</v>
+        <v>-0.20245078944536879</v>
       </c>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.2">
@@ -6031,21 +6031,21 @@
         <f>J37</f>
         <v>0</v>
       </c>
-      <c r="D26" s="33" t="e">
+      <c r="D26" s="33">
         <f>K37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E26" s="33" t="e">
+        <v>-0.57903681911096483</v>
+      </c>
+      <c r="E26" s="33">
         <f>L37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F26" s="33" t="e">
+        <v>-0.3943306525851169</v>
+      </c>
+      <c r="F26" s="33">
         <f>M37</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G26" s="33" t="e">
+        <v>-0.20319232197177453</v>
+      </c>
+      <c r="G26" s="33">
         <f>N37</f>
-        <v>#REF!</v>
+        <v>-4.5351682239474958E-2</v>
       </c>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.2">
@@ -6055,21 +6055,21 @@
       <c r="C27" s="26">
         <v>0</v>
       </c>
-      <c r="D27" s="34" t="e">
+      <c r="D27" s="34">
         <f>K49</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E27" s="34" t="e">
+        <v>-0.43045596379246831</v>
+      </c>
+      <c r="E27" s="34">
         <f t="shared" ref="E27:G27" si="4">L49</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F27" s="34" t="e">
+        <v>-0.18915885187210035</v>
+      </c>
+      <c r="F27" s="34">
         <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G27" s="34" t="e">
+        <v>-0.17100234100196271</v>
+      </c>
+      <c r="G27" s="34">
         <f t="shared" si="4"/>
-        <v>#REF!</v>
+        <v>-0.14149246034975063</v>
       </c>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.2">
@@ -6096,25 +6096,25 @@
       <c r="I30" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="J30" s="14" t="e">
-        <f>SUM(summary!#REF!)/SUM(summary!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K30" s="14" t="e">
-        <f>SUM(summary!#REF!)/SUM(summary!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L30" s="14" t="e">
-        <f>SUM(summary!#REF!)/SUM(summary!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M30" s="14" t="e">
-        <f>SUM(summary!#REF!)/SUM(summary!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N30" s="14" t="e">
-        <f>SUM(summary!#REF!)/SUM(summary!#REF!)</f>
-        <v>#REF!</v>
+      <c r="J30" s="14">
+        <f>SUM(summary!C$13:C$15)/SUM(summary!$H$13:$H$15)</f>
+        <v>4.8658444901393587E-2</v>
+      </c>
+      <c r="K30" s="14">
+        <f>SUM(summary!D$13:D$15)/SUM(summary!$H$13:$H$15)</f>
+        <v>0.282971286887164</v>
+      </c>
+      <c r="L30" s="14">
+        <f>SUM(summary!E$13:E$15)/SUM(summary!$H$13:$H$15)</f>
+        <v>0.37561800158327896</v>
+      </c>
+      <c r="M30" s="14">
+        <f>SUM(summary!F$13:F$15)/SUM(summary!$H$13:$H$15)</f>
+        <v>0.17798943484906571</v>
+      </c>
+      <c r="N30" s="14">
+        <f>SUM(summary!G$13:G$15)/SUM(summary!$H$13:$H$15)</f>
+        <v>0.11476283177909773</v>
       </c>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.2">
@@ -6146,50 +6146,50 @@
       <c r="I32" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J32" s="14" t="e">
+      <c r="J32" s="14">
         <f>J31-J30</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K32" s="14" t="e">
+        <v>0.15134155509860642</v>
+      </c>
+      <c r="K32" s="14">
         <f>K31-K30</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L32" s="14" t="e">
+        <v>-8.2971286887163986E-2</v>
+      </c>
+      <c r="L32" s="14">
         <f>L31-L30</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M32" s="14" t="e">
+        <v>-0.17561800158327895</v>
+      </c>
+      <c r="M32" s="14">
         <f>M31-M30</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N32" s="14" t="e">
+        <v>2.2010565150934303E-2</v>
+      </c>
+      <c r="N32" s="14">
         <f>N31-N30</f>
-        <v>#REF!</v>
+        <v>8.5237168220902285E-2</v>
       </c>
     </row>
     <row r="33" spans="9:14" x14ac:dyDescent="0.2">
       <c r="I33" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="J33" s="16" t="e">
+      <c r="J33" s="16">
         <f>J32/J30</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K33" s="16" t="e">
+        <v>3.1102834339506802</v>
+      </c>
+      <c r="K33" s="16">
         <f>K32/K30</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L33" s="16" t="e">
+        <v>-0.29321450879307459</v>
+      </c>
+      <c r="L33" s="16">
         <f>L32/L30</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M33" s="16" t="e">
+        <v>-0.46754415614540867</v>
+      </c>
+      <c r="M33" s="16">
         <f>M32/M30</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N33" s="16" t="e">
+        <v>0.1236622003412684</v>
+      </c>
+      <c r="N33" s="16">
         <f>N32/N30</f>
-        <v>#REF!</v>
+        <v>0.74272451193058586</v>
       </c>
     </row>
     <row r="34" spans="9:14" x14ac:dyDescent="0.2">
@@ -6230,21 +6230,21 @@
       <c r="J36" s="19">
         <v>0</v>
       </c>
-      <c r="K36" s="20" t="e">
+      <c r="K36" s="20">
         <f>damp*LN(K30/K31)-damp*LN($J30/$J31)-K11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L36" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="L36" s="20">
         <f>damp*LN(L30/L31)-damp*LN($J30/$J31)-L11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M36" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="M36" s="20">
         <f>damp*LN(M30/M31)-damp*LN($J30/$J31)-M11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N36" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="N36" s="20">
         <f>damp*LN(N30/N31)-damp*LN($J30/$J31)</f>
-        <v>#REF!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="9:14" x14ac:dyDescent="0.2">
@@ -6255,21 +6255,21 @@
         <f>J35+J36</f>
         <v>0</v>
       </c>
-      <c r="K37" s="21" t="e">
+      <c r="K37" s="21">
         <f>K35+K36</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L37" s="21" t="e">
+        <v>-0.57903681911096483</v>
+      </c>
+      <c r="L37" s="21">
         <f>L35+L36</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M37" s="21" t="e">
+        <v>-0.3943306525851169</v>
+      </c>
+      <c r="M37" s="21">
         <f>M35+M36</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N37" s="21" t="e">
+        <v>-0.20319232197177453</v>
+      </c>
+      <c r="N37" s="21">
         <f>N35+N36</f>
-        <v>#REF!</v>
+        <v>-4.5351682239474958E-2</v>
       </c>
     </row>
     <row r="41" spans="9:14" x14ac:dyDescent="0.2">
@@ -6296,25 +6296,25 @@
       <c r="I42" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="J42" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K42" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L42" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M42" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N42" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
+      <c r="J42" s="14">
+        <f>summary!C30</f>
+        <v>4.0705456263286352E-2</v>
+      </c>
+      <c r="K42" s="14">
+        <f>summary!D30</f>
+        <v>0.32342925753877649</v>
+      </c>
+      <c r="L42" s="14">
+        <f>summary!E30</f>
+        <v>0.42723998110385009</v>
+      </c>
+      <c r="M42" s="14">
+        <f>summary!F30</f>
+        <v>0.1584225651523502</v>
+      </c>
+      <c r="N42" s="14">
+        <f>summary!G30</f>
+        <v>5.0202739941736872E-2</v>
       </c>
     </row>
     <row r="43" spans="9:14" x14ac:dyDescent="0.2">
@@ -6346,50 +6346,50 @@
       <c r="I44" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J44" s="14" t="e">
+      <c r="J44" s="14">
         <f>J43-J42</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K44" s="14" t="e">
+        <v>0.15929454373671365</v>
+      </c>
+      <c r="K44" s="14">
         <f>K43-K42</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L44" s="14" t="e">
+        <v>-0.12342925753877648</v>
+      </c>
+      <c r="L44" s="14">
         <f>L43-L42</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M44" s="14" t="e">
+        <v>-0.22723998110385007</v>
+      </c>
+      <c r="M44" s="14">
         <f>M43-M42</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N44" s="14" t="e">
+        <v>4.1577434847649808E-2</v>
+      </c>
+      <c r="N44" s="14">
         <f>N43-N42</f>
-        <v>#REF!</v>
+        <v>0.14979726005826313</v>
       </c>
     </row>
     <row r="45" spans="9:14" x14ac:dyDescent="0.2">
       <c r="I45" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="J45" s="16" t="e">
+      <c r="J45" s="16">
         <f>J44/J42</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K45" s="16" t="e">
+        <v>3.9133462282398455</v>
+      </c>
+      <c r="K45" s="16">
         <f>K44/K42</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L45" s="16" t="e">
+        <v>-0.38162675349176883</v>
+      </c>
+      <c r="L45" s="16">
         <f>L44/L42</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M45" s="16" t="e">
+        <v>-0.53187901683905003</v>
+      </c>
+      <c r="M45" s="16">
         <f>M44/M42</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N45" s="16" t="e">
+        <v>0.26244641858731454</v>
+      </c>
+      <c r="N45" s="16">
         <f>N44/N42</f>
-        <v>#REF!</v>
+        <v>2.9838463046461476</v>
       </c>
     </row>
     <row r="46" spans="9:14" x14ac:dyDescent="0.2">
@@ -6430,21 +6430,21 @@
       <c r="J48" s="19">
         <v>0</v>
       </c>
-      <c r="K48" s="20" t="e">
+      <c r="K48" s="20">
         <f>damp*LN(K42/K43)-damp*LN($J42/$J43)-K11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L48" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="L48" s="20">
         <f>damp*LN(L42/L43)-damp*LN($J42/$J43)-L11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M48" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="M48" s="20">
         <f>damp*LN(M42/M43)-damp*LN($J42/$J43)-M11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N48" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="N48" s="20">
         <f>damp*LN(N42/N43)-damp*LN($J42/$J43)-N11</f>
-        <v>#REF!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="9:14" x14ac:dyDescent="0.2">
@@ -6455,21 +6455,21 @@
         <f>J47+J48</f>
         <v>0</v>
       </c>
-      <c r="K49" s="21" t="e">
+      <c r="K49" s="21">
         <f>K47+K48</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L49" s="21" t="e">
+        <v>-0.43045596379246831</v>
+      </c>
+      <c r="L49" s="21">
         <f>L47+L48</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M49" s="21" t="e">
+        <v>-0.18915885187210035</v>
+      </c>
+      <c r="M49" s="21">
         <f>M47+M48</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N49" s="21" t="e">
+        <v>-0.17100234100196271</v>
+      </c>
+      <c r="N49" s="21">
         <f>N47+N48</f>
-        <v>#REF!</v>
+        <v>-0.14149246034975063</v>
       </c>
     </row>
     <row r="52" spans="9:14" x14ac:dyDescent="0.2">
@@ -6499,25 +6499,25 @@
       <c r="I54" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="J54" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K54" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L54" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M54" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N54" s="14" t="e">
-        <f>summary!#REF!</f>
-        <v>#REF!</v>
+      <c r="J54" s="14">
+        <f>summary!C24</f>
+        <v>5.8864185807506283E-2</v>
+      </c>
+      <c r="K54" s="14">
+        <f>summary!D24</f>
+        <v>0.32659954413574355</v>
+      </c>
+      <c r="L54" s="14">
+        <f>summary!E24</f>
+        <v>0.37599635789400931</v>
+      </c>
+      <c r="M54" s="14">
+        <f>summary!F24</f>
+        <v>0.15005506732036258</v>
+      </c>
+      <c r="N54" s="14">
+        <f>summary!G24</f>
+        <v>8.8484844842378244E-2</v>
       </c>
     </row>
     <row r="55" spans="9:14" x14ac:dyDescent="0.2">
@@ -6549,50 +6549,50 @@
       <c r="I56" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J56" s="14" t="e">
+      <c r="J56" s="14">
         <f>J55-J54</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K56" s="14" t="e">
+        <v>0.14113581419249371</v>
+      </c>
+      <c r="K56" s="14">
         <f>K55-K54</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L56" s="14" t="e">
+        <v>-0.12659954413574354</v>
+      </c>
+      <c r="L56" s="14">
         <f>L55-L54</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M56" s="14" t="e">
+        <v>-0.1759963578940093</v>
+      </c>
+      <c r="M56" s="14">
         <f>M55-M54</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N56" s="14" t="e">
+        <v>4.9944932679637427E-2</v>
+      </c>
+      <c r="N56" s="14">
         <f>N55-N54</f>
-        <v>#REF!</v>
+        <v>0.11151515515762177</v>
       </c>
     </row>
     <row r="57" spans="9:14" x14ac:dyDescent="0.2">
       <c r="I57" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="J57" s="16" t="e">
+      <c r="J57" s="16">
         <f>J56/J54</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K57" s="16" t="e">
+        <v>2.3976516833856598</v>
+      </c>
+      <c r="K57" s="16">
         <f>K56/K54</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L57" s="16" t="e">
+        <v>-0.38762927385815749</v>
+      </c>
+      <c r="L57" s="16">
         <f>L56/L54</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M57" s="16" t="e">
+        <v>-0.46807995396493018</v>
+      </c>
+      <c r="M57" s="16">
         <f>M56/M54</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N57" s="16" t="e">
+        <v>0.33284402567363258</v>
+      </c>
+      <c r="N57" s="16">
         <f>N56/N54</f>
-        <v>#REF!</v>
+        <v>1.2602740656467035</v>
       </c>
     </row>
     <row r="58" spans="9:14" x14ac:dyDescent="0.2">
@@ -6633,21 +6633,21 @@
       <c r="J60" s="19">
         <v>0</v>
       </c>
-      <c r="K60" s="20" t="e">
+      <c r="K60" s="20">
         <f>damp*LN(K54/K55)-damp*LN($J54/$J55)-K11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L60" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="L60" s="20">
         <f>damp*LN(L54/L55)-damp*LN($J54/$J55)-L11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M60" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="M60" s="20">
         <f>damp*LN(M54/M55)-damp*LN($J54/$J55)-M11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N60" s="20" t="e">
+        <v>0</v>
+      </c>
+      <c r="N60" s="20">
         <f>damp*LN(N54/N55)-damp*LN($J54/$J55)-N11</f>
-        <v>#REF!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="9:14" x14ac:dyDescent="0.2">
@@ -6658,21 +6658,21 @@
         <f>J59+J60</f>
         <v>0</v>
       </c>
-      <c r="K61" s="21" t="e">
+      <c r="K61" s="21">
         <f>K59+K60</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L61" s="21" t="e">
+        <v>0.1844471057264194</v>
+      </c>
+      <c r="L61" s="21">
         <f>L59+L60</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M61" s="21" t="e">
+        <v>0.1844471057264194</v>
+      </c>
+      <c r="M61" s="21">
         <f>M59+M60</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N61" s="21" t="e">
+        <v>0.20643155178083641</v>
+      </c>
+      <c r="N61" s="21">
         <f>N59+N60</f>
-        <v>#REF!</v>
+        <v>0.20643155178083641</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correct the cell references for the constants
</commit_message>
<xml_diff>
--- a/utilities/calibration/workbook_templates/02_AutoOwnership_2023_blank.xlsx
+++ b/utilities/calibration/workbook_templates/02_AutoOwnership_2023_blank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one\utilities\calibration\workbook_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC053FE-9649-4243-AAD0-DA750F063B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6462C0E4-C99B-47D0-B0DF-28E8E4C85F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1476" yWindow="8556" windowWidth="26460" windowHeight="13560" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="3" r:id="rId1"/>
@@ -25,7 +25,7 @@
   <definedNames>
     <definedName name="damp">calibration!$J$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcOnSave="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -3137,116 +3137,122 @@
       <sheetName val="Auto Time"/>
       <sheetName val="Transit Time"/>
       <sheetName val="Walk Time"/>
-      <sheetName val="Calibration"/>
-      <sheetName val="Calibration (3 futures)"/>
+      <sheetName val="CalibrationRunsBlueprint (2035)"/>
+      <sheetName val="CalibrationRunsBlueprint"/>
+      <sheetName val="CalibrationTargets_Blueprint"/>
+      <sheetName val="CalibrationTargets_RSGexample"/>
+      <sheetName val="CalibrationTargets_3futures"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="0"/>
       <sheetData sheetId="1">
         <row r="53">
           <cell r="H53">
-            <v>1.1172992162790916</v>
+            <v>0.97594798926411408</v>
           </cell>
           <cell r="J53">
-            <v>-1.2565051850306308</v>
+            <v>-1.519233909162766</v>
           </cell>
           <cell r="M53">
-            <v>-3.3877106944960214</v>
+            <v>-3.5560350664680063</v>
           </cell>
           <cell r="Q53">
-            <v>-5.3502031433147499</v>
+            <v>-5.3109685729222527</v>
           </cell>
         </row>
         <row r="54">
           <cell r="H54">
-            <v>0.57931801393948956</v>
+            <v>0.38650670107434598</v>
           </cell>
           <cell r="J54">
-            <v>0.56301198136124597</v>
+            <v>0.51732584823260019</v>
           </cell>
           <cell r="M54">
-            <v>0.4050938414636639</v>
+            <v>0.32605968644578215</v>
           </cell>
           <cell r="Q54">
-            <v>-0.20245078944536879</v>
+            <v>-1.6844385041155208E-2</v>
           </cell>
         </row>
         <row r="55">
           <cell r="H55">
-            <v>-0.57903681911096483</v>
+            <v>-0.43524342980119346</v>
           </cell>
           <cell r="J55">
-            <v>-0.3943306525851169</v>
+            <v>-0.15603857443089025</v>
           </cell>
           <cell r="M55">
-            <v>-0.20319232197177453</v>
+            <v>5.6263830423431277E-2</v>
           </cell>
           <cell r="Q55">
-            <v>-4.5351682239474958E-2</v>
+            <v>0.30446760983612964</v>
           </cell>
         </row>
         <row r="56">
           <cell r="H56">
-            <v>-0.57903681911096483</v>
+            <v>-0.43524342980119346</v>
           </cell>
           <cell r="J56">
-            <v>-0.3943306525851169</v>
+            <v>-0.15603857443089025</v>
           </cell>
           <cell r="M56">
-            <v>-0.20319232197177453</v>
+            <v>5.6263830423431277E-2</v>
           </cell>
           <cell r="Q56">
-            <v>-4.5351682239474958E-2</v>
+            <v>0.30446760983612964</v>
           </cell>
         </row>
         <row r="57">
           <cell r="H57">
-            <v>-0.57903681911096483</v>
+            <v>-0.43524342980119346</v>
           </cell>
           <cell r="J57">
-            <v>-0.3943306525851169</v>
+            <v>-0.15603857443089025</v>
           </cell>
           <cell r="M57">
-            <v>-0.20319232197177453</v>
+            <v>5.6263830423431277E-2</v>
           </cell>
           <cell r="Q57">
-            <v>-4.5351682239474958E-2</v>
+            <v>0.30446760983612964</v>
           </cell>
         </row>
         <row r="58">
           <cell r="H58">
-            <v>-0.43045596379246831</v>
+            <v>-0.22547748611134263</v>
           </cell>
           <cell r="J58">
-            <v>-0.18915885187210035</v>
+            <v>-3.2893536624987285E-2</v>
           </cell>
           <cell r="M58">
-            <v>-0.17100234100196271</v>
+            <v>6.0685059579343448E-3</v>
           </cell>
           <cell r="Q58">
-            <v>-0.14149246034975063</v>
+            <v>-0.42549225622244535</v>
           </cell>
         </row>
         <row r="59">
           <cell r="H59">
-            <v>0.1844471057264194</v>
-          </cell>
-          <cell r="I59">
-            <v>0.1844471057264194</v>
+            <v>0.25725032285672278</v>
           </cell>
           <cell r="J59">
-            <v>0.20643155178083641</v>
+            <v>0.28463037247556472</v>
           </cell>
-          <cell r="K59">
-            <v>0.20643155178083641</v>
+          <cell r="M59">
+            <v>0.30819475462611823</v>
+          </cell>
+          <cell r="Q59">
+            <v>0.30740373277725497</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3520,28 +3526,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:X31"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" style="1" customWidth="1"/>
-    <col min="3" max="7" width="9.140625" style="1"/>
-    <col min="8" max="8" width="10.85546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" style="1"/>
-    <col min="10" max="10" width="14.5703125" style="1" customWidth="1"/>
-    <col min="11" max="12" width="9.140625" style="1"/>
+    <col min="2" max="2" width="14.5546875" style="1" customWidth="1"/>
+    <col min="3" max="7" width="9.109375" style="1"/>
+    <col min="8" max="8" width="10.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="1"/>
+    <col min="10" max="10" width="14.5546875" style="1" customWidth="1"/>
+    <col min="11" max="12" width="9.109375" style="1"/>
     <col min="13" max="13" width="10" style="1" customWidth="1"/>
-    <col min="14" max="15" width="9.140625" style="1"/>
-    <col min="16" max="16" width="10.28515625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="1"/>
-    <col min="18" max="18" width="13.140625" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="1"/>
+    <col min="14" max="15" width="9.109375" style="1"/>
+    <col min="16" max="16" width="10.33203125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="9.109375" style="1"/>
+    <col min="18" max="18" width="13.109375" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="13"/>
       <c r="B2" s="13"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="35" t="s">
         <v>189</v>
       </c>
@@ -3552,10 +3558,10 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="13"/>
     </row>
-    <row r="6" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13"/>
       <c r="B6" s="4" t="s">
         <v>29</v>
@@ -3580,7 +3586,7 @@
       <c r="O6" s="40"/>
       <c r="P6" s="40"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="13"/>
       <c r="C7" s="5">
         <v>0</v>
@@ -3619,7 +3625,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
       <c r="B8" s="6" t="s">
         <v>19</v>
@@ -3676,7 +3682,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>
       <c r="B9" s="6" t="s">
         <v>20</v>
@@ -3733,7 +3739,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>
       <c r="B10" s="6" t="s">
         <v>21</v>
@@ -3790,7 +3796,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="13"/>
       <c r="B11" s="6" t="s">
         <v>22</v>
@@ -3847,7 +3853,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
       <c r="B12" s="6" t="s">
         <v>23</v>
@@ -3904,7 +3910,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>
       <c r="B13" s="6" t="s">
         <v>24</v>
@@ -3961,7 +3967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="6" t="s">
         <v>25</v>
@@ -4018,7 +4024,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="6" t="s">
         <v>26</v>
@@ -4075,7 +4081,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>
       <c r="B16" s="7" t="s">
         <v>27</v>
@@ -4132,7 +4138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A17" s="13"/>
       <c r="B17" s="6" t="s">
         <v>28</v>
@@ -4189,7 +4195,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A18" s="13"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -4198,10 +4204,10 @@
       <c r="G18" s="8"/>
       <c r="R18" s="35"/>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A19" s="13"/>
     </row>
-    <row r="20" spans="1:24" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="13"/>
       <c r="B20" s="4" t="s">
         <v>29</v>
@@ -4237,7 +4243,7 @@
       <c r="W20" s="40"/>
       <c r="X20" s="40"/>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21" s="13"/>
       <c r="C21" s="5">
         <v>0</v>
@@ -4294,7 +4300,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A22" s="13"/>
       <c r="B22" s="6" t="s">
         <v>19</v>
@@ -4378,7 +4384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>
       <c r="B23" s="6" t="s">
         <v>20</v>
@@ -4462,7 +4468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A24" s="13"/>
       <c r="B24" s="6" t="s">
         <v>21</v>
@@ -4546,7 +4552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A25" s="13"/>
       <c r="B25" s="6" t="s">
         <v>22</v>
@@ -4630,7 +4636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A26" s="13"/>
       <c r="B26" s="6" t="s">
         <v>23</v>
@@ -4714,7 +4720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A27" s="13"/>
       <c r="B27" s="6" t="s">
         <v>24</v>
@@ -4798,7 +4804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A28" s="13"/>
       <c r="B28" s="6" t="s">
         <v>25</v>
@@ -4882,7 +4888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A29" s="13"/>
       <c r="B29" s="6" t="s">
         <v>26</v>
@@ -4966,7 +4972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A30" s="13"/>
       <c r="B30" s="7" t="s">
         <v>27</v>
@@ -5050,7 +5056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A31" s="13"/>
       <c r="B31" s="6" t="s">
         <v>28</v>
@@ -5186,17 +5192,17 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:N61"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" style="1" customWidth="1"/>
-    <col min="3" max="8" width="9.140625" style="1"/>
-    <col min="9" max="9" width="20.140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" style="1" customWidth="1"/>
+    <col min="3" max="8" width="9.109375" style="1"/>
+    <col min="9" max="9" width="20.109375" style="1" customWidth="1"/>
     <col min="10" max="14" width="9" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="1"/>
+    <col min="15" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.3">
       <c r="I1" s="1" t="s">
         <v>57</v>
       </c>
@@ -5204,7 +5210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B4" s="27" t="s">
         <v>33</v>
       </c>
@@ -5242,7 +5248,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B5" s="29" t="s">
         <v>39</v>
       </c>
@@ -5250,20 +5256,20 @@
         <v>0</v>
       </c>
       <c r="D5" s="33">
-        <f>'[1]Auto ownership'!H53</f>
-        <v>1.1172992162790916</v>
+        <f>'[1]Auto ownership'!$H$53</f>
+        <v>0.97594798926411408</v>
       </c>
       <c r="E5" s="33">
-        <f>'[1]Auto ownership'!J53</f>
-        <v>-1.2565051850306308</v>
+        <f>'[1]Auto ownership'!$J$53</f>
+        <v>-1.519233909162766</v>
       </c>
       <c r="F5" s="33">
-        <f>'[1]Auto ownership'!M53</f>
-        <v>-3.3877106944960214</v>
+        <f>'[1]Auto ownership'!$M$53</f>
+        <v>-3.5560350664680063</v>
       </c>
       <c r="G5" s="33">
-        <f>'[1]Auto ownership'!Q53</f>
-        <v>-5.3502031433147499</v>
+        <f>'[1]Auto ownership'!$Q$53</f>
+        <v>-5.3109685729222527</v>
       </c>
       <c r="I5" s="22" t="s">
         <v>40</v>
@@ -5289,7 +5295,7 @@
         <v>8.1515180632999756E-2</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B6" s="30" t="s">
         <v>41</v>
       </c>
@@ -5297,20 +5303,20 @@
         <v>0</v>
       </c>
       <c r="D6" s="33">
-        <f>'[1]Auto ownership'!H54</f>
-        <v>0.57931801393948956</v>
+        <f>'[1]Auto ownership'!$H$54</f>
+        <v>0.38650670107434598</v>
       </c>
       <c r="E6" s="33">
-        <f>'[1]Auto ownership'!J54</f>
-        <v>0.56301198136124597</v>
+        <f>'[1]Auto ownership'!$J$54</f>
+        <v>0.51732584823260019</v>
       </c>
       <c r="F6" s="33">
-        <f>'[1]Auto ownership'!M54</f>
-        <v>0.4050938414636639</v>
+        <f>'[1]Auto ownership'!$M$54</f>
+        <v>0.32605968644578215</v>
       </c>
       <c r="G6" s="33">
-        <f>'[1]Auto ownership'!Q54</f>
-        <v>-0.20245078944536879</v>
+        <f>'[1]Auto ownership'!$Q$54</f>
+        <v>-1.6844385041155208E-2</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>42</v>
@@ -5336,7 +5342,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B7" s="15" t="s">
         <v>43</v>
       </c>
@@ -5379,7 +5385,7 @@
         <v>0.11848481936700025</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B8" s="15" t="s">
         <v>45</v>
       </c>
@@ -5387,20 +5393,20 @@
         <v>0</v>
       </c>
       <c r="D8" s="33">
-        <f>'[1]Auto ownership'!H59</f>
-        <v>0.1844471057264194</v>
+        <f>'[1]Auto ownership'!$H$59</f>
+        <v>0.25725032285672278</v>
       </c>
       <c r="E8" s="33">
-        <f>'[1]Auto ownership'!I59</f>
-        <v>0.1844471057264194</v>
+        <f>'[1]Auto ownership'!$J$59</f>
+        <v>0.28463037247556472</v>
       </c>
       <c r="F8" s="33">
-        <f>'[1]Auto ownership'!J59</f>
-        <v>0.20643155178083641</v>
+        <f>'[1]Auto ownership'!$M$59</f>
+        <v>0.30819475462611823</v>
       </c>
       <c r="G8" s="33">
-        <f>'[1]Auto ownership'!K59</f>
-        <v>0.20643155178083641</v>
+        <f>'[1]Auto ownership'!$Q$59</f>
+        <v>0.30740373277725497</v>
       </c>
       <c r="I8" s="18" t="s">
         <v>46</v>
@@ -5426,7 +5432,7 @@
         <v>1.4535307220926907</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="15" t="s">
         <v>47</v>
       </c>
@@ -5454,7 +5460,7 @@
       <c r="M9" s="19"/>
       <c r="N9" s="19"/>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10" s="15" t="s">
         <v>48</v>
       </c>
@@ -5482,22 +5488,22 @@
       </c>
       <c r="K10" s="23">
         <f>D5</f>
-        <v>1.1172992162790916</v>
+        <v>0.97594798926411408</v>
       </c>
       <c r="L10" s="23">
         <f t="shared" ref="L10:N10" si="2">E5</f>
-        <v>-1.2565051850306308</v>
+        <v>-1.519233909162766</v>
       </c>
       <c r="M10" s="23">
         <f t="shared" si="2"/>
-        <v>-3.3877106944960214</v>
+        <v>-3.5560350664680063</v>
       </c>
       <c r="N10" s="23">
         <f t="shared" si="2"/>
-        <v>-5.3502031433147499</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.2">
+        <v>-5.3109685729222527</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11" s="15" t="s">
         <v>49</v>
       </c>
@@ -5505,20 +5511,20 @@
         <v>0</v>
       </c>
       <c r="D11" s="33">
-        <f>'[1]Auto ownership'!H55</f>
-        <v>-0.57903681911096483</v>
+        <f>'[1]Auto ownership'!$H$55</f>
+        <v>-0.43524342980119346</v>
       </c>
       <c r="E11" s="33">
-        <f>'[1]Auto ownership'!J55</f>
-        <v>-0.3943306525851169</v>
+        <f>'[1]Auto ownership'!$J$55</f>
+        <v>-0.15603857443089025</v>
       </c>
       <c r="F11" s="33">
-        <f>'[1]Auto ownership'!M55</f>
-        <v>-0.20319232197177453</v>
+        <f>'[1]Auto ownership'!$M$55</f>
+        <v>5.6263830423431277E-2</v>
       </c>
       <c r="G11" s="33">
-        <f>'[1]Auto ownership'!Q55</f>
-        <v>-4.5351682239474958E-2</v>
+        <f>'[1]Auto ownership'!$Q$55</f>
+        <v>0.30446760983612964</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>53</v>
@@ -5543,7 +5549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" s="15" t="s">
         <v>50</v>
       </c>
@@ -5551,20 +5557,20 @@
         <v>0</v>
       </c>
       <c r="D12" s="33">
-        <f>'[1]Auto ownership'!H56</f>
-        <v>-0.57903681911096483</v>
+        <f>'[1]Auto ownership'!$H$56</f>
+        <v>-0.43524342980119346</v>
       </c>
       <c r="E12" s="33">
-        <f>'[1]Auto ownership'!J56</f>
-        <v>-0.3943306525851169</v>
+        <f>'[1]Auto ownership'!$J$56</f>
+        <v>-0.15603857443089025</v>
       </c>
       <c r="F12" s="33">
-        <f>'[1]Auto ownership'!M56</f>
-        <v>-0.20319232197177453</v>
+        <f>'[1]Auto ownership'!$M$56</f>
+        <v>5.6263830423431277E-2</v>
       </c>
       <c r="G12" s="33">
-        <f>'[1]Auto ownership'!Q56</f>
-        <v>-4.5351682239474958E-2</v>
+        <f>'[1]Auto ownership'!$Q$56</f>
+        <v>0.30446760983612964</v>
       </c>
       <c r="I12" s="18" t="s">
         <v>59</v>
@@ -5575,22 +5581,22 @@
       </c>
       <c r="K12" s="21">
         <f>K10+K11</f>
-        <v>1.1172992162790916</v>
+        <v>0.97594798926411408</v>
       </c>
       <c r="L12" s="21">
         <f>L10+L11</f>
-        <v>-1.2565051850306308</v>
+        <v>-1.519233909162766</v>
       </c>
       <c r="M12" s="21">
         <f>M10+M11</f>
-        <v>-3.3877106944960214</v>
+        <v>-3.5560350664680063</v>
       </c>
       <c r="N12" s="21">
         <f>N10+N11</f>
-        <v>-5.3502031433147499</v>
-      </c>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
+        <v>-5.3109685729222527</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13" s="15" t="s">
         <v>51</v>
       </c>
@@ -5598,23 +5604,23 @@
         <v>0</v>
       </c>
       <c r="D13" s="33">
-        <f>'[1]Auto ownership'!H57</f>
-        <v>-0.57903681911096483</v>
+        <f>'[1]Auto ownership'!$H$57</f>
+        <v>-0.43524342980119346</v>
       </c>
       <c r="E13" s="33">
-        <f>'[1]Auto ownership'!J57</f>
-        <v>-0.3943306525851169</v>
+        <f>'[1]Auto ownership'!$J$57</f>
+        <v>-0.15603857443089025</v>
       </c>
       <c r="F13" s="33">
-        <f>'[1]Auto ownership'!M57</f>
-        <v>-0.20319232197177453</v>
+        <f>'[1]Auto ownership'!$M$57</f>
+        <v>5.6263830423431277E-2</v>
       </c>
       <c r="G13" s="33">
-        <f>'[1]Auto ownership'!Q57</f>
-        <v>-4.5351682239474958E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
+        <f>'[1]Auto ownership'!$Q$57</f>
+        <v>0.30446760983612964</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="31" t="s">
         <v>52</v>
       </c>
@@ -5622,23 +5628,23 @@
         <v>0</v>
       </c>
       <c r="D14" s="34">
-        <f>'[1]Auto ownership'!H58</f>
-        <v>-0.43045596379246831</v>
+        <f>'[1]Auto ownership'!$H$58</f>
+        <v>-0.22547748611134263</v>
       </c>
       <c r="E14" s="34">
-        <f>'[1]Auto ownership'!J58</f>
-        <v>-0.18915885187210035</v>
+        <f>'[1]Auto ownership'!$J$58</f>
+        <v>-3.2893536624987285E-2</v>
       </c>
       <c r="F14" s="34">
-        <f>'[1]Auto ownership'!M58</f>
-        <v>-0.17100234100196271</v>
+        <f>'[1]Auto ownership'!$M$58</f>
+        <v>6.0685059579343448E-3</v>
       </c>
       <c r="G14" s="34">
-        <f>'[1]Auto ownership'!Q58</f>
-        <v>-0.14149246034975063</v>
-      </c>
-    </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.2">
+        <f>'[1]Auto ownership'!$Q$58</f>
+        <v>-0.42549225622244535</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B17" s="27" t="s">
         <v>54</v>
       </c>
@@ -5676,7 +5682,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>39</v>
       </c>
@@ -5685,19 +5691,19 @@
       </c>
       <c r="D18" s="33">
         <f>K12</f>
-        <v>1.1172992162790916</v>
+        <v>0.97594798926411408</v>
       </c>
       <c r="E18" s="33">
         <f>L12</f>
-        <v>-1.2565051850306308</v>
+        <v>-1.519233909162766</v>
       </c>
       <c r="F18" s="33">
         <f>M12</f>
-        <v>-3.3877106944960214</v>
+        <v>-3.5560350664680063</v>
       </c>
       <c r="G18" s="33">
         <f>N12</f>
-        <v>-5.3502031433147499</v>
+        <v>-5.3109685729222527</v>
       </c>
       <c r="I18" s="22" t="s">
         <v>40</v>
@@ -5723,7 +5729,7 @@
         <v>2.1183946326476303E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B19" s="30" t="s">
         <v>41</v>
       </c>
@@ -5732,19 +5738,19 @@
       </c>
       <c r="D19" s="33">
         <f>K25</f>
-        <v>0.57931801393948956</v>
+        <v>0.38650670107434598</v>
       </c>
       <c r="E19" s="33">
         <f>L25</f>
-        <v>0.56301198136124597</v>
+        <v>0.51732584823260019</v>
       </c>
       <c r="F19" s="33">
         <f>M25</f>
-        <v>0.4050938414636639</v>
+        <v>0.32605968644578215</v>
       </c>
       <c r="G19" s="33">
         <f>N25</f>
-        <v>-0.20245078944536879</v>
+        <v>-1.6844385041155208E-2</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>42</v>
@@ -5770,7 +5776,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B20" s="15" t="s">
         <v>43</v>
       </c>
@@ -5813,7 +5819,7 @@
         <v>0.17881605367352371</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B21" s="15" t="s">
         <v>45</v>
       </c>
@@ -5823,19 +5829,19 @@
       </c>
       <c r="D21" s="33">
         <f>K61</f>
-        <v>0.1844471057264194</v>
+        <v>0.25725032285672278</v>
       </c>
       <c r="E21" s="33">
         <f t="shared" ref="E21:G21" si="3">L61</f>
-        <v>0.1844471057264194</v>
+        <v>0.28463037247556472</v>
       </c>
       <c r="F21" s="33">
         <f t="shared" si="3"/>
-        <v>0.20643155178083641</v>
+        <v>0.30819475462611823</v>
       </c>
       <c r="G21" s="33">
         <f t="shared" si="3"/>
-        <v>0.20643155178083641</v>
+        <v>0.30740373277725497</v>
       </c>
       <c r="I21" s="18" t="s">
         <v>46</v>
@@ -5861,7 +5867,7 @@
         <v>8.4411115340692824</v>
       </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B22" s="15" t="s">
         <v>47</v>
       </c>
@@ -5885,7 +5891,7 @@
       <c r="L22" s="14"/>
       <c r="M22" s="14"/>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B23" s="15" t="s">
         <v>48</v>
       </c>
@@ -5913,22 +5919,22 @@
       </c>
       <c r="K23" s="23">
         <f>D6</f>
-        <v>0.57931801393948956</v>
+        <v>0.38650670107434598</v>
       </c>
       <c r="L23" s="23">
         <f>E6</f>
-        <v>0.56301198136124597</v>
+        <v>0.51732584823260019</v>
       </c>
       <c r="M23" s="23">
         <f>F6</f>
-        <v>0.4050938414636639</v>
+        <v>0.32605968644578215</v>
       </c>
       <c r="N23" s="23">
         <f>G6</f>
-        <v>-0.20245078944536879</v>
-      </c>
-    </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.2">
+        <v>-1.6844385041155208E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B24" s="15" t="s">
         <v>49</v>
       </c>
@@ -5938,19 +5944,19 @@
       </c>
       <c r="D24" s="33">
         <f>K37</f>
-        <v>-0.57903681911096483</v>
+        <v>-0.43524342980119346</v>
       </c>
       <c r="E24" s="33">
         <f>L37</f>
-        <v>-0.3943306525851169</v>
+        <v>-0.15603857443089025</v>
       </c>
       <c r="F24" s="33">
         <f>M37</f>
-        <v>-0.20319232197177453</v>
+        <v>5.6263830423431277E-2</v>
       </c>
       <c r="G24" s="33">
         <f>N37</f>
-        <v>-4.5351682239474958E-2</v>
+        <v>0.30446760983612964</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>53</v>
@@ -5975,7 +5981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B25" s="15" t="s">
         <v>50</v>
       </c>
@@ -5985,19 +5991,19 @@
       </c>
       <c r="D25" s="33">
         <f>K37</f>
-        <v>-0.57903681911096483</v>
+        <v>-0.43524342980119346</v>
       </c>
       <c r="E25" s="33">
         <f>L37</f>
-        <v>-0.3943306525851169</v>
+        <v>-0.15603857443089025</v>
       </c>
       <c r="F25" s="33">
         <f>M37</f>
-        <v>-0.20319232197177453</v>
+        <v>5.6263830423431277E-2</v>
       </c>
       <c r="G25" s="33">
         <f>N37</f>
-        <v>-4.5351682239474958E-2</v>
+        <v>0.30446760983612964</v>
       </c>
       <c r="I25" s="18" t="s">
         <v>59</v>
@@ -6008,22 +6014,22 @@
       </c>
       <c r="K25" s="21">
         <f>K23+K24</f>
-        <v>0.57931801393948956</v>
+        <v>0.38650670107434598</v>
       </c>
       <c r="L25" s="21">
         <f>L23+L24</f>
-        <v>0.56301198136124597</v>
+        <v>0.51732584823260019</v>
       </c>
       <c r="M25" s="21">
         <f>M23+M24</f>
-        <v>0.4050938414636639</v>
+        <v>0.32605968644578215</v>
       </c>
       <c r="N25" s="21">
         <f>N23+N24</f>
-        <v>-0.20245078944536879</v>
-      </c>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.2">
+        <v>-1.6844385041155208E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B26" s="15" t="s">
         <v>51</v>
       </c>
@@ -6033,22 +6039,22 @@
       </c>
       <c r="D26" s="33">
         <f>K37</f>
-        <v>-0.57903681911096483</v>
+        <v>-0.43524342980119346</v>
       </c>
       <c r="E26" s="33">
         <f>L37</f>
-        <v>-0.3943306525851169</v>
+        <v>-0.15603857443089025</v>
       </c>
       <c r="F26" s="33">
         <f>M37</f>
-        <v>-0.20319232197177453</v>
+        <v>5.6263830423431277E-2</v>
       </c>
       <c r="G26" s="33">
         <f>N37</f>
-        <v>-4.5351682239474958E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.2">
+        <v>0.30446760983612964</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B27" s="31" t="s">
         <v>52</v>
       </c>
@@ -6057,22 +6063,22 @@
       </c>
       <c r="D27" s="34">
         <f>K49</f>
-        <v>-0.43045596379246831</v>
+        <v>-0.22547748611134263</v>
       </c>
       <c r="E27" s="34">
         <f t="shared" ref="E27:G27" si="4">L49</f>
-        <v>-0.18915885187210035</v>
+        <v>-3.2893536624987285E-2</v>
       </c>
       <c r="F27" s="34">
         <f t="shared" si="4"/>
-        <v>-0.17100234100196271</v>
+        <v>6.0685059579343448E-3</v>
       </c>
       <c r="G27" s="34">
         <f t="shared" si="4"/>
-        <v>-0.14149246034975063</v>
-      </c>
-    </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.2">
+        <v>-0.42549225622244535</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
       <c r="I29" s="27" t="s">
         <v>55</v>
       </c>
@@ -6092,7 +6098,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
       <c r="I30" s="22" t="s">
         <v>40</v>
       </c>
@@ -6117,7 +6123,7 @@
         <v>0.11476283177909773</v>
       </c>
     </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:14" x14ac:dyDescent="0.3">
       <c r="I31" s="1" t="s">
         <v>42</v>
       </c>
@@ -6142,7 +6148,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:14" x14ac:dyDescent="0.3">
       <c r="I32" s="1" t="s">
         <v>44</v>
       </c>
@@ -6167,7 +6173,7 @@
         <v>8.5237168220902285E-2</v>
       </c>
     </row>
-    <row r="33" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I33" s="18" t="s">
         <v>46</v>
       </c>
@@ -6192,13 +6198,13 @@
         <v>0.74272451193058586</v>
       </c>
     </row>
-    <row r="34" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="9:14" x14ac:dyDescent="0.3">
       <c r="J34" s="14"/>
       <c r="K34" s="14"/>
       <c r="L34" s="14"/>
       <c r="M34" s="14"/>
     </row>
-    <row r="35" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I35" s="22" t="s">
         <v>58</v>
       </c>
@@ -6208,22 +6214,22 @@
       </c>
       <c r="K35" s="23">
         <f>D12</f>
-        <v>-0.57903681911096483</v>
+        <v>-0.43524342980119346</v>
       </c>
       <c r="L35" s="23">
         <f>E12</f>
-        <v>-0.3943306525851169</v>
+        <v>-0.15603857443089025</v>
       </c>
       <c r="M35" s="23">
         <f>F12</f>
-        <v>-0.20319232197177453</v>
+        <v>5.6263830423431277E-2</v>
       </c>
       <c r="N35" s="23">
         <f>G12</f>
-        <v>-4.5351682239474958E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="9:14" x14ac:dyDescent="0.2">
+        <v>0.30446760983612964</v>
+      </c>
+    </row>
+    <row r="36" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I36" s="1" t="s">
         <v>53</v>
       </c>
@@ -6247,7 +6253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="37" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I37" s="18" t="s">
         <v>59</v>
       </c>
@@ -6257,22 +6263,22 @@
       </c>
       <c r="K37" s="21">
         <f>K35+K36</f>
-        <v>-0.57903681911096483</v>
+        <v>-0.43524342980119346</v>
       </c>
       <c r="L37" s="21">
         <f>L35+L36</f>
-        <v>-0.3943306525851169</v>
+        <v>-0.15603857443089025</v>
       </c>
       <c r="M37" s="21">
         <f>M35+M36</f>
-        <v>-0.20319232197177453</v>
+        <v>5.6263830423431277E-2</v>
       </c>
       <c r="N37" s="21">
         <f>N35+N36</f>
-        <v>-4.5351682239474958E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="9:14" x14ac:dyDescent="0.2">
+        <v>0.30446760983612964</v>
+      </c>
+    </row>
+    <row r="41" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I41" s="27" t="s">
         <v>27</v>
       </c>
@@ -6292,7 +6298,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="42" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I42" s="22" t="s">
         <v>40</v>
       </c>
@@ -6317,7 +6323,7 @@
         <v>5.0202739941736872E-2</v>
       </c>
     </row>
-    <row r="43" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="43" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I43" s="1" t="s">
         <v>42</v>
       </c>
@@ -6342,7 +6348,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="44" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="44" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I44" s="1" t="s">
         <v>44</v>
       </c>
@@ -6367,7 +6373,7 @@
         <v>0.14979726005826313</v>
       </c>
     </row>
-    <row r="45" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="45" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I45" s="18" t="s">
         <v>46</v>
       </c>
@@ -6392,13 +6398,13 @@
         <v>2.9838463046461476</v>
       </c>
     </row>
-    <row r="46" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="46" spans="9:14" x14ac:dyDescent="0.3">
       <c r="J46" s="14"/>
       <c r="K46" s="14"/>
       <c r="L46" s="14"/>
       <c r="M46" s="14"/>
     </row>
-    <row r="47" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="47" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I47" s="22" t="s">
         <v>58</v>
       </c>
@@ -6408,22 +6414,22 @@
       </c>
       <c r="K47" s="23">
         <f>D14</f>
-        <v>-0.43045596379246831</v>
+        <v>-0.22547748611134263</v>
       </c>
       <c r="L47" s="23">
         <f>E14</f>
-        <v>-0.18915885187210035</v>
+        <v>-3.2893536624987285E-2</v>
       </c>
       <c r="M47" s="23">
         <f>F14</f>
-        <v>-0.17100234100196271</v>
+        <v>6.0685059579343448E-3</v>
       </c>
       <c r="N47" s="23">
         <f>G14</f>
-        <v>-0.14149246034975063</v>
-      </c>
-    </row>
-    <row r="48" spans="9:14" x14ac:dyDescent="0.2">
+        <v>-0.42549225622244535</v>
+      </c>
+    </row>
+    <row r="48" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I48" s="1" t="s">
         <v>53</v>
       </c>
@@ -6447,7 +6453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="49" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I49" s="18" t="s">
         <v>59</v>
       </c>
@@ -6457,25 +6463,25 @@
       </c>
       <c r="K49" s="21">
         <f>K47+K48</f>
-        <v>-0.43045596379246831</v>
+        <v>-0.22547748611134263</v>
       </c>
       <c r="L49" s="21">
         <f>L47+L48</f>
-        <v>-0.18915885187210035</v>
+        <v>-3.2893536624987285E-2</v>
       </c>
       <c r="M49" s="21">
         <f>M47+M48</f>
-        <v>-0.17100234100196271</v>
+        <v>6.0685059579343448E-3</v>
       </c>
       <c r="N49" s="21">
         <f>N47+N48</f>
-        <v>-0.14149246034975063</v>
-      </c>
-    </row>
-    <row r="52" spans="9:14" x14ac:dyDescent="0.2">
+        <v>-0.42549225622244535</v>
+      </c>
+    </row>
+    <row r="52" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I52" s="13"/>
     </row>
-    <row r="53" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="53" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I53" s="27" t="s">
         <v>21</v>
       </c>
@@ -6495,7 +6501,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="54" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I54" s="22" t="s">
         <v>40</v>
       </c>
@@ -6520,7 +6526,7 @@
         <v>8.8484844842378244E-2</v>
       </c>
     </row>
-    <row r="55" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="55" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I55" s="1" t="s">
         <v>42</v>
       </c>
@@ -6545,7 +6551,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="56" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="56" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I56" s="1" t="s">
         <v>44</v>
       </c>
@@ -6570,7 +6576,7 @@
         <v>0.11151515515762177</v>
       </c>
     </row>
-    <row r="57" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="57" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I57" s="18" t="s">
         <v>46</v>
       </c>
@@ -6595,13 +6601,13 @@
         <v>1.2602740656467035</v>
       </c>
     </row>
-    <row r="58" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="58" spans="9:14" x14ac:dyDescent="0.3">
       <c r="J58" s="14"/>
       <c r="K58" s="14"/>
       <c r="L58" s="14"/>
       <c r="M58" s="14"/>
     </row>
-    <row r="59" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="59" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I59" s="22" t="s">
         <v>58</v>
       </c>
@@ -6611,22 +6617,22 @@
       </c>
       <c r="K59" s="23">
         <f>D8</f>
-        <v>0.1844471057264194</v>
+        <v>0.25725032285672278</v>
       </c>
       <c r="L59" s="23">
         <f>E8</f>
-        <v>0.1844471057264194</v>
+        <v>0.28463037247556472</v>
       </c>
       <c r="M59" s="23">
         <f>F8</f>
-        <v>0.20643155178083641</v>
+        <v>0.30819475462611823</v>
       </c>
       <c r="N59" s="23">
         <f>G8</f>
-        <v>0.20643155178083641</v>
-      </c>
-    </row>
-    <row r="60" spans="9:14" x14ac:dyDescent="0.2">
+        <v>0.30740373277725497</v>
+      </c>
+    </row>
+    <row r="60" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I60" s="1" t="s">
         <v>53</v>
       </c>
@@ -6650,7 +6656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="61" spans="9:14" x14ac:dyDescent="0.3">
       <c r="I61" s="18" t="s">
         <v>59</v>
       </c>
@@ -6660,19 +6666,19 @@
       </c>
       <c r="K61" s="21">
         <f>K59+K60</f>
-        <v>0.1844471057264194</v>
+        <v>0.25725032285672278</v>
       </c>
       <c r="L61" s="21">
         <f>L59+L60</f>
-        <v>0.1844471057264194</v>
+        <v>0.28463037247556472</v>
       </c>
       <c r="M61" s="21">
         <f>M59+M60</f>
-        <v>0.20643155178083641</v>
+        <v>0.30819475462611823</v>
       </c>
       <c r="N61" s="21">
         <f>N59+N60</f>
-        <v>0.20643155178083641</v>
+        <v>0.30740373277725497</v>
       </c>
     </row>
   </sheetData>
@@ -6735,23 +6741,23 @@
     <tabColor theme="6"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
@@ -6774,7 +6780,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -6797,7 +6803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>2</v>
       </c>
@@ -6820,7 +6826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -6843,7 +6849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>4</v>
       </c>
@@ -6866,7 +6872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>5</v>
       </c>
@@ -6889,7 +6895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>6</v>
       </c>
@@ -6912,7 +6918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>7</v>
       </c>
@@ -6935,7 +6941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>8</v>
       </c>
@@ -6958,7 +6964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>9</v>
       </c>
@@ -6992,85 +6998,85 @@
     <tabColor theme="4"/>
   </sheetPr>
   <dimension ref="A1:BK15"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="1"/>
-    <col min="3" max="3" width="28.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="1"/>
+    <col min="1" max="1" width="16.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="1"/>
+    <col min="3" max="3" width="28.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" style="1"/>
     <col min="5" max="5" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="1"/>
+    <col min="16" max="16" width="9.109375" style="1"/>
     <col min="17" max="17" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="9.140625" style="1"/>
+    <col min="18" max="18" width="9.109375" style="1"/>
     <col min="19" max="19" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="9.140625" style="1"/>
+    <col min="20" max="20" width="9.109375" style="1"/>
     <col min="21" max="21" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="9.140625" style="1"/>
+    <col min="22" max="22" width="9.109375" style="1"/>
     <col min="23" max="23" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="9.140625" style="1"/>
+    <col min="24" max="24" width="9.109375" style="1"/>
     <col min="25" max="25" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="9.140625" style="1"/>
+    <col min="26" max="26" width="9.109375" style="1"/>
     <col min="27" max="27" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="9.140625" style="1"/>
+    <col min="28" max="28" width="9.109375" style="1"/>
     <col min="29" max="29" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="9.140625" style="1"/>
+    <col min="30" max="30" width="9.109375" style="1"/>
     <col min="31" max="31" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="32" max="32" width="9.140625" style="1"/>
+    <col min="32" max="32" width="9.109375" style="1"/>
     <col min="33" max="33" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="9.140625" style="1"/>
+    <col min="34" max="34" width="9.109375" style="1"/>
     <col min="35" max="35" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="36" max="36" width="9.140625" style="1"/>
+    <col min="36" max="36" width="9.109375" style="1"/>
     <col min="37" max="37" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="38" max="38" width="9.140625" style="1"/>
+    <col min="38" max="38" width="9.109375" style="1"/>
     <col min="39" max="39" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="40" max="40" width="9.140625" style="1"/>
+    <col min="40" max="40" width="9.109375" style="1"/>
     <col min="41" max="41" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="42" max="42" width="9.140625" style="1"/>
+    <col min="42" max="42" width="9.109375" style="1"/>
     <col min="43" max="43" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="44" max="44" width="9.140625" style="1"/>
+    <col min="44" max="44" width="9.109375" style="1"/>
     <col min="45" max="45" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="46" max="46" width="9.140625" style="1"/>
+    <col min="46" max="46" width="9.109375" style="1"/>
     <col min="47" max="47" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="48" max="48" width="9.140625" style="1"/>
+    <col min="48" max="48" width="9.109375" style="1"/>
     <col min="49" max="49" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="50" max="50" width="9.140625" style="1"/>
+    <col min="50" max="50" width="9.109375" style="1"/>
     <col min="51" max="51" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="52" max="52" width="9.140625" style="1"/>
+    <col min="52" max="52" width="9.109375" style="1"/>
     <col min="53" max="53" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="54" max="54" width="9.140625" style="1"/>
+    <col min="54" max="54" width="9.109375" style="1"/>
     <col min="55" max="55" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="56" max="56" width="9.140625" style="1"/>
+    <col min="56" max="56" width="9.109375" style="1"/>
     <col min="57" max="57" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="58" max="58" width="9.140625" style="1"/>
+    <col min="58" max="58" width="9.109375" style="1"/>
     <col min="59" max="59" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="60" max="60" width="9.140625" style="1"/>
+    <col min="60" max="60" width="9.109375" style="1"/>
     <col min="61" max="61" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="62" max="62" width="9.140625" style="1"/>
+    <col min="62" max="62" width="9.109375" style="1"/>
     <col min="63" max="63" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="64" max="16384" width="9.140625" style="1"/>
+    <col min="64" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="2" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="3" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>62</v>
       </c>
@@ -7261,7 +7267,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:63" s="2" customFormat="1" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:63" s="2" customFormat="1" ht="138" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -7452,7 +7458,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -7643,7 +7649,7 @@
         <v>2675</v>
       </c>
     </row>
-    <row r="6" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -7834,7 +7840,7 @@
         <v>3017</v>
       </c>
     </row>
-    <row r="7" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -8025,7 +8031,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="8" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -8216,7 +8222,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="9" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -8407,7 +8413,7 @@
         <v>1381</v>
       </c>
     </row>
-    <row r="10" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -8598,7 +8604,7 @@
         <v>1909</v>
       </c>
     </row>
-    <row r="11" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
@@ -8789,7 +8795,7 @@
         <v>2903</v>
       </c>
     </row>
-    <row r="12" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>15</v>
       </c>
@@ -8980,7 +8986,7 @@
         <v>1612</v>
       </c>
     </row>
-    <row r="13" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>17</v>
       </c>
@@ -9171,7 +9177,7 @@
         <v>2141</v>
       </c>
     </row>
-    <row r="15" spans="1:63" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:63" x14ac:dyDescent="0.3">
       <c r="F15" s="1">
         <v>0</v>
       </c>

</xml_diff>